<commit_message>
Actualizar Excel, PowerPoint y diagramas con los datos del informe
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P9bj8o7UcwbCu86Zsog7Lb
</commit_message>
<xml_diff>
--- a/Actividad Alva instructora Luna de Cristal/2_Paso2_Matriz_de_analisis.xlsx
+++ b/Actividad Alva instructora Luna de Cristal/2_Paso2_Matriz_de_analisis.xlsx
@@ -476,14 +476,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fuente: observación directa y conversación con la dueña de Luna de Cristal (Yopal), octubre de 2026. Ajusta cualquier dato que no corresponda a la realidad.</t>
+          <t>Fuente: informe del proyecto (entrevista a la propietaria 24/06/2026; encuestas a 2 colaboradores, 45 clientas y 5 proveedores) y diagnóstico propio. Elaboración propia.</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="62" customHeight="1">
+    <row r="5" ht="64" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Situaciones que afectan el desempeño</t>
@@ -541,22 +541,22 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Pocas clientas nuevas llegan a la tienda.</t>
+          <t>Bajo alcance en redes sociales y ausencia en Google Maps.</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Redes inactivas y negocio ausente en Google Maps.</t>
+          <t>Publicaciones sin estrategia y perfil de Maps sin crear.</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Ventas bajas y dependencia de clientas que ya conocen el local.</t>
+          <t>Pocas clientas nuevas; dependencia de las que ya conocen la tienda.</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Perfil de Google Maps, WhatsApp Business y contenido diario.</t>
+          <t>Perfil de Google Maps, catálogo en WhatsApp Business y contenido constante con fotos y videos.</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -565,7 +565,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="62" customHeight="1">
+    <row r="6" ht="64" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Situaciones que afectan el desempeño</t>
@@ -573,12 +573,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Prendas sin rotación durante meses.</t>
+          <t>Prendas con baja rotación.</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Compras sin análisis de lo que se vende y sin promociones.</t>
+          <t>Compras sin datos de lo que más se vende.</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -597,7 +597,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="62" customHeight="1">
+    <row r="7" ht="64" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Factores que limitan la innovación</t>
@@ -605,249 +605,281 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Se trabaja "como siempre se ha hecho".</t>
+          <t>Procesos manuales: sin POS, facturación ni inventario sistematizado.</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Falta de tiempo y desconocimiento de herramientas digitales.</t>
+          <t>Costos de la tecnología y negocio en etapa de introducción.</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>El negocio no aprovecha medios gratuitos para vender.</t>
+          <t>Pérdida de datos y demoras en la atención.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Capacitar a la dueña en herramientas simples y apoyarse en el aprendiz.</t>
+          <t>Implementar por etapas: hoja de cálculo primero, luego POS y facturación electrónica.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="64" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Factores que limitan la innovación</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Equipo de solo dos personas.</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>La propietaria compra, vende y maneja redes.</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Poco tiempo para planear e innovar.</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Repartir tareas y usar herramientas gratuitas e IA para el contenido.</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
           <t>Media</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="62" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Factores que limitan la innovación</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Presupuesto muy limitado.</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Ingresos ajustados.</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Miedo a probar ideas nuevas.</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Usar herramientas gratuitas y probar ideas pequeñas antes de invertir.</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
+    <row r="9" ht="64" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Aspectos administrativos susceptibles de mejora</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Valores, políticas y organigrama desconocidos (0 %).</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Cultura organizacional sin documentar.</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Identidad poco clara para el equipo.</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Documentar organigrama, valores y manual de funciones e incluirlos en la inducción.</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="62" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="10" ht="64" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Aspectos administrativos susceptibles de mejora</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>No hay registro de ventas ni de indicadores.</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Procesos informales y manejo "de memoria".</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>No se sabe qué funciona ni qué se vende más.</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Hoja de registro diaria: mensajes, ventas, ganancia y origen de la clienta.</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>No hay indicadores de ventas ni plan comercial.</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Registros informales.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Decisiones improvisadas y riesgo de descuentos con pérdida.</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Registro diario (ventas, mensajes, origen de la clienta, reseñas) y plan de 30 días con descuento máximo.</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="62" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Aspectos administrativos susceptibles de mejora</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>No hay plan comercial ni reglas de descuento.</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Decisiones improvisadas.</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Riesgo de descuentos que generan pérdida.</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Plan de 30 días y descuento máximo de 15-20 % en prendas y 10 % en perfumes.</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
+    <row r="11" ht="64" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Necesidades de clientes internos</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>El 100 % pide mejorar la tecnología.</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Herramientas actuales limitadas para el control.</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Más trabajo manual y errores.</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Portafolio digital y sistema de inventario sencillo.</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="64" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Necesidades de clientes externos</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Las clientas quieren estilo, buen precio y atención cercana; cada vez compran más por redes.</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Los hábitos de compra se movieron a lo digital.</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Si no encuentran la tienda en línea, compran en otro lugar.</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Catálogo digital con precios, respuesta rápida por WhatsApp y domicilio.</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="64" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Necesidades de proveedores</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Comunicación innovadora y retroalimentación solo "algunas veces" (60 %).</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Comunicación solo por WhatsApp (100 %).</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Menor coordinación en pedidos.</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Enviar retroalimentación periódica y planear compras con datos de ventas.</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="62" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Necesidades de clientes internos</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>La dueña necesita apoyo con lo digital y tiempo para atender.</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Todo el trabajo recae en una persona.</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Agotamiento y tareas sin hacer.</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Repartir tareas: el aprendiz maneja redes, fotos y métricas.</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
+    <row r="14" ht="64" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Oportunidades de crecimiento</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Mercado en crecimiento impulsado por el comercio digital.</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Cambio de hábitos de las clientas.</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Posibilidad de llegar a más clientas sin abrir otro local.</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Portafolio digital, Meta Ads segmentado y campañas de temporada.</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="62" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Necesidades de clientes externos</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Las clientas quieren ver productos y precios antes de ir, y respuesta rápida.</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>No hay catálogo digital ni respuesta oportuna.</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Clientas que se van a la competencia.</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Catálogo en WhatsApp Business, respuestas rápidas y fotos con precio.</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="62" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="15" ht="64" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Oportunidades de crecimiento</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Temporadas comerciales sin aprovechar.</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>No hay calendario comercial.</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Se pierden las épocas de más ventas.</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Campañas de Halloween, Black Friday y diciembre (perfumes como regalo).</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="62" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Oportunidades de crecimiento</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Herramientas de IA gratuitas o de bajo costo.</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Avance tecnológico reciente.</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Contenido profesional sin pagar agencia.</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>Mejorar fotos y crear videos publicitarios con IA; luego automatizar mensajes.</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Fotos mejoradas y videos publicitarios con IA; luego automatizar mensajes.</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
@@ -870,14 +902,14 @@
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Diagrama causa-efecto en tabla – Efecto: ventas por debajo de su potencial</t>
+          <t>Causa-efecto en tabla – Efecto: ventas por debajo de su potencial</t>
         </is>
       </c>
     </row>
@@ -918,7 +950,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Redes sociales inactivas</t>
+          <t>Bajo alcance en redes sociales</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -928,7 +960,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Sin promociones planeadas</t>
+          <t>Sin calendario de promociones</t>
         </is>
       </c>
     </row>
@@ -940,17 +972,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Mensajes sin respuesta rápida</t>
+          <t>Sin sistema POS ni facturación</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Sin WhatsApp Business</t>
+          <t>Inventario llevado a mano</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Procesos informales</t>
+          <t>Funciones sin documentar</t>
         </is>
       </c>
     </row>
@@ -962,12 +994,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>No se registran ventas diarias</t>
+          <t>Ventas sin registro digital</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>No se sabe de dónde llegan las clientas</t>
+          <t>No se sabe qué se vende más ni qué queda quieto</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -984,17 +1016,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Prendas quietas por meses</t>
+          <t>Prendas con baja rotación</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Dinero parado en inventario</t>
+          <t>Poca variedad de perfumes y correas</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Poca rotación por temporada</t>
+          <t>Espacio reducido en el local</t>
         </is>
       </c>
     </row>
@@ -1006,17 +1038,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Poco tiempo para lo digital</t>
+          <t>Equipo de solo 2 personas</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Desconocimiento de herramientas digitales</t>
+          <t>Valores y organigrama desconocidos (0 %)</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Todo recae en la dueña</t>
+          <t>Todo recae en la propietaria</t>
         </is>
       </c>
     </row>
@@ -1028,12 +1060,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Competencia de otras tiendas en Yopal</t>
+          <t>Competencia con más trayectoria en Yopal</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Compras por internet</t>
+          <t>Lluvias, inflación e IVA</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Corregir dueño y personal de Luna de Cristal en todos los archivos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P9bj8o7UcwbCu86Zsog7Lb
</commit_message>
<xml_diff>
--- a/Actividad Alva instructora Luna de Cristal/2_Paso2_Matriz_de_analisis.xlsx
+++ b/Actividad Alva instructora Luna de Cristal/2_Paso2_Matriz_de_analisis.xlsx
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fuente: informe del proyecto (entrevista a la propietaria 24/06/2026; encuestas a 2 colaboradores, 45 clientas y 5 proveedores) y diagnóstico propio. Elaboración propia.</t>
+          <t>Fuente: informe del proyecto (entrevista a la dirección del negocio 24/06/2026; encuestas a 2 colaboradores, 45 clientas y 5 proveedores) y diagnóstico propio. Elaboración propia.</t>
         </is>
       </c>
     </row>
@@ -637,12 +637,12 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Equipo de solo dos personas.</t>
+          <t>Equipo pequeño: la administradora y una prima.</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>La propietaria compra, vende y maneja redes.</t>
+          <t>La administradora compra, atiende y maneja redes.</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Todo recae en la propietaria</t>
+          <t>Todo recae en la administradora</t>
         </is>
       </c>
     </row>

</xml_diff>